<commit_message>
Agregar tienda e-commerce con Stripe: carrito, checkout, pedidos
</commit_message>
<xml_diff>
--- a/distribucion/excel_analisis_datos/codigos/c05_tendencias/ventas_historicas.xlsx
+++ b/distribucion/excel_analisis_datos/codigos/c05_tendencias/ventas_historicas.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2023-01-04</t>
+          <t>2023-02-12</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -496,21 +496,21 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>2982.92</v>
+        <v>4735.13</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2023-01-24</t>
+          <t>2023-02-23</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -524,54 +524,54 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>123052.74</v>
+        <v>48680.79</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2023-01-14</t>
+          <t>2023-03-05</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>13608.99</v>
+        <v>42614.67</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2023-01-02</t>
+          <t>2023-03-21</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -580,38 +580,38 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>4411.74</v>
+        <v>30657.92</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2023-01-28</t>
+          <t>2023-04-28</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>2800.91</v>
+        <v>3018.06</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -622,12 +622,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2023-02-12</t>
+          <t>2023-04-04</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -636,26 +636,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>11492.59</v>
+        <v>13645.68</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2023-02-03</t>
+          <t>2023-04-12</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -664,10 +664,10 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>33454.74</v>
+        <v>8900.969999999999</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -678,63 +678,63 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2023-02-26</t>
+          <t>2023-05-27</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1450.05</v>
+        <v>9491.74</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2023-02-03</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>2686.23</v>
+        <v>30840.39</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2023-03-25</t>
+          <t>2023-05-26</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -748,26 +748,26 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>98156.34</v>
+        <v>137389.97</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2023-03-05</t>
+          <t>2023-05-28</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -776,82 +776,82 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>4536.19</v>
+        <v>8946.040000000001</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2023-04-01</t>
+          <t>2023-05-26</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>5441.23</v>
+        <v>8870.65</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2023-04-06</t>
+          <t>2023-06-16</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>5670.79</v>
+        <v>16911.64</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2023-04-04</t>
+          <t>2023-06-02</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -860,54 +860,54 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>164504.06</v>
+        <v>7529.5</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2023-04-17</t>
+          <t>2023-07-25</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>44009.27</v>
+        <v>13948.04</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2023-04-02</t>
+          <t>2023-07-17</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -916,10 +916,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>14897.64</v>
+        <v>83584.44</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -930,24 +930,24 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2023-05-02</t>
+          <t>2023-07-16</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>2309.41</v>
+        <v>4845.75</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -958,12 +958,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2023-05-16</t>
+          <t>2023-08-02</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -972,54 +972,54 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>9747.190000000001</v>
+        <v>13895.87</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2023-05-05</t>
+          <t>2023-08-28</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>2148.76</v>
+        <v>29725.22</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2023-05-13</t>
+          <t>2023-08-11</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1028,110 +1028,110 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>4945.16</v>
+        <v>26256.7</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2023-06-04</t>
+          <t>2023-08-21</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>28794.44</v>
+        <v>9757.280000000001</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2023-06-25</t>
+          <t>2023-09-15</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>148711.31</v>
+        <v>13167.62</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2023-06-14</t>
+          <t>2023-09-16</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>22065.53</v>
+        <v>10700.29</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2023-06-14</t>
+          <t>2023-09-18</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1140,26 +1140,26 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>4331.27</v>
+        <v>43201.63</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2023-07-03</t>
+          <t>2023-09-21</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1168,26 +1168,26 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>30711.01</v>
+        <v>10570.12</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2023-07-26</t>
+          <t>2023-09-22</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1196,26 +1196,26 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>31114.38</v>
+        <v>8207.48</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2023-07-18</t>
+          <t>2023-10-25</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1227,23 +1227,23 @@
         <v>40</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>9659.290000000001</v>
+        <v>49149.68</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2023-07-25</t>
+          <t>2023-10-23</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1252,10 +1252,10 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>8329.610000000001</v>
+        <v>6933.55</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1266,40 +1266,40 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2023-08-10</t>
+          <t>2023-10-01</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>14603.46</v>
+        <v>3311.49</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2023-08-22</t>
+          <t>2023-11-23</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1308,54 +1308,54 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>11857.61</v>
+        <v>11607.93</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2023-08-25</t>
+          <t>2023-11-24</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>13762.28</v>
+        <v>57698.23</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2023-08-25</t>
+          <t>2023-11-15</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1364,49 +1364,49 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>10636.85</v>
+        <v>4408.73</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2023-08-01</t>
+          <t>2023-12-25</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>7356.95</v>
+        <v>4816.18</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2023-09-12</t>
+          <t>2023-12-22</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1420,26 +1420,26 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>74981.60000000001</v>
+        <v>143315.14</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2023-09-03</t>
+          <t>2023-12-24</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1448,21 +1448,21 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>33421.5</v>
+        <v>11144</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2023-09-14</t>
+          <t>2023-12-17</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1476,10 +1476,10 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>5171.61</v>
+        <v>8555.35</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -1490,12 +1490,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2023-10-20</t>
+          <t>2024-01-24</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1504,10 +1504,10 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>31957.15</v>
+        <v>4464.81</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -1518,12 +1518,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>2024-01-17</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1532,10 +1532,10 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>8796.639999999999</v>
+        <v>68881.8</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -1546,12 +1546,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2023-10-20</t>
+          <t>2024-01-25</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1560,94 +1560,94 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>8895.68</v>
+        <v>44443.52</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2023-11-14</t>
+          <t>2024-01-15</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>11296.68</v>
+        <v>4774.32</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2023-11-10</t>
+          <t>2024-01-24</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>47135.98</v>
+        <v>7037.26</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2023-11-01</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>30108.31</v>
+        <v>15219.43</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -1658,12 +1658,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2023-11-10</t>
+          <t>2024-02-22</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -1672,26 +1672,26 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>31286.23</v>
+        <v>55817.78</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2023-11-06</t>
+          <t>2024-02-06</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -1700,26 +1700,26 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>9489.83</v>
+        <v>43233.64</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2023-11-18</t>
+          <t>2024-02-18</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -1728,66 +1728,66 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>9216.040000000001</v>
+        <v>5229.39</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2023-12-14</t>
+          <t>2024-02-14</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>6913.67</v>
+        <v>7450.91</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2023-12-14</t>
+          <t>2024-03-17</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>172089.72</v>
+        <v>4698.6</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -1798,12 +1798,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2023-12-06</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -1812,26 +1812,26 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>8482.120000000001</v>
+        <v>27720.98</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2023-12-12</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -1840,10 +1840,10 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>10405.88</v>
+        <v>14403.93</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -1854,68 +1854,68 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2024-01-03</t>
+          <t>2024-03-07</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>24968.41</v>
+        <v>5484.75</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2024-01-11</t>
+          <t>2024-04-28</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>50679.53</v>
+        <v>50150.85</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2024-01-17</t>
+          <t>2024-04-18</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -1924,26 +1924,26 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>10821.5</v>
+        <v>184604.36</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2024-01-27</t>
+          <t>2024-04-10</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>6023.41</v>
+        <v>78517.19</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -1966,12 +1966,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-04-14</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -1980,26 +1980,26 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>107761.45</v>
+        <v>10094.9</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2024-02-25</t>
+          <t>2024-04-01</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2008,38 +2008,38 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>39010.31</v>
+        <v>1887.72</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>2024-02-11</t>
+          <t>2024-05-27</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>9387.43</v>
+        <v>10916.02</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -2050,7 +2050,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2024-03-26</t>
+          <t>2024-05-24</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2064,21 +2064,21 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>25162.53</v>
+        <v>33835.46</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2024-03-02</t>
+          <t>2024-05-06</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -2092,21 +2092,21 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>2190.93</v>
+        <v>4188.06</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2024-04-20</t>
+          <t>2024-06-09</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -2120,21 +2120,21 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>4635.61</v>
+        <v>12964.19</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>2024-04-26</t>
+          <t>2024-06-11</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -2148,26 +2148,26 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>46312.06</v>
+        <v>4221.38</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2024-04-21</t>
+          <t>2024-06-02</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -2176,10 +2176,10 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>159025.08</v>
+        <v>54424.18</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -2190,12 +2190,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2024-04-02</t>
+          <t>2024-06-16</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -2204,54 +2204,54 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>21386.26</v>
+        <v>6347.89</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2024-04-17</t>
+          <t>2024-07-17</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>3344.98</v>
+        <v>8259.93</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>2024-05-17</t>
+          <t>2024-07-06</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -2260,21 +2260,21 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>11602.55</v>
+        <v>30921.21</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2024-05-14</t>
+          <t>2024-07-08</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2288,26 +2288,26 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>97894.07000000001</v>
+        <v>93025.10000000001</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>2024-05-03</t>
+          <t>2024-07-17</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -2316,10 +2316,10 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>6278.6</v>
+        <v>7880.17</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -2330,40 +2330,40 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-08-01</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>4325.25</v>
+        <v>14859.4</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>2024-06-03</t>
+          <t>2024-08-20</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -2372,10 +2372,10 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>9250.59</v>
+        <v>42373.51</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -2386,40 +2386,40 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2024-06-21</t>
+          <t>2024-08-11</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>21209.8</v>
+        <v>149955.77</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>2024-06-10</t>
+          <t>2024-08-01</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -2428,10 +2428,10 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>12141.41</v>
+        <v>6223.04</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -2442,12 +2442,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>2024-06-23</t>
+          <t>2024-08-15</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -2456,21 +2456,21 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>12523.05</v>
+        <v>6642.42</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>2024-07-12</t>
+          <t>2024-09-11</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -2484,26 +2484,26 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>11702.22</v>
+        <v>5966.53</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2024-07-07</t>
+          <t>2024-09-18</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -2512,122 +2512,122 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>40837.33</v>
+        <v>112502.97</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>2024-08-25</t>
+          <t>2024-09-28</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>13053.01</v>
+        <v>4666.86</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>2024-08-20</t>
+          <t>2024-10-21</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>15215.37</v>
+        <v>11909.53</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>2024-08-26</t>
+          <t>2024-10-01</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>8557.809999999999</v>
+        <v>11802.96</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>2024-09-20</t>
+          <t>2024-11-14</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>101057.68</v>
+        <v>22436.07</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -2638,12 +2638,12 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>2024-09-27</t>
+          <t>2024-11-13</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -2652,10 +2652,10 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>5914.46</v>
+        <v>23176.38</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -2666,96 +2666,96 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2024-10-25</t>
+          <t>2024-11-25</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>11380.62</v>
+        <v>2885.27</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>2024-10-06</t>
+          <t>2024-11-12</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>28020.02</v>
+        <v>2149.51</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2024-10-18</t>
+          <t>2024-12-03</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>7608.01</v>
+        <v>44707.19</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>2024-10-03</t>
+          <t>2024-12-16</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -2764,21 +2764,21 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>4357.86</v>
+        <v>7822.62</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2024-11-05</t>
+          <t>2025-01-10</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2792,54 +2792,54 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>17912.32</v>
+        <v>11848.49</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>2024-11-27</t>
+          <t>2025-01-12</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>20200.6</v>
+        <v>125738.3</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2024-11-02</t>
+          <t>2025-01-05</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -2848,21 +2848,21 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>125349.22</v>
+        <v>35506.45</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>2024-11-08</t>
+          <t>2025-01-18</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -2876,10 +2876,10 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>8150.74</v>
+        <v>6057.03</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -2890,68 +2890,68 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2024-11-11</t>
+          <t>2025-02-07</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>11238.89</v>
+        <v>7221.6</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>2024-12-23</t>
+          <t>2025-02-07</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>40783</v>
+        <v>17720.15</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>2024-12-03</t>
+          <t>2025-02-15</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -2960,26 +2960,26 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>17352.97</v>
+        <v>8231.48</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>2024-12-24</t>
+          <t>2025-03-11</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -2988,26 +2988,26 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>63758.82</v>
+        <v>142994.15</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>2025-01-15</t>
+          <t>2025-03-11</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -3016,26 +3016,26 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>102206.88</v>
+        <v>5484.45</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>2025-01-21</t>
+          <t>2025-03-23</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -3044,38 +3044,38 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>4814.76</v>
+        <v>5673.93</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2025-01-14</t>
+          <t>2025-04-14</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>4051.41</v>
+        <v>10457.75</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -3086,40 +3086,40 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>2025-02-22</t>
+          <t>2025-04-09</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E95" s="3" t="n">
-        <v>11876.74</v>
+        <v>52546.68</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2025-02-26</t>
+          <t>2025-04-16</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -3128,26 +3128,26 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>101863.43</v>
+        <v>8188.7</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>2025-02-21</t>
+          <t>2025-04-18</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -3156,38 +3156,38 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>1221.72</v>
+        <v>7632.23</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>2025-03-08</t>
+          <t>2025-05-07</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>31136</v>
+        <v>118890.34</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -3198,12 +3198,12 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>2025-03-05</t>
+          <t>2025-05-28</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -3212,21 +3212,21 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>95976.37</v>
+        <v>7210.34</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>2025-03-15</t>
+          <t>2025-05-13</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -3240,21 +3240,21 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="E100" s="3" t="n">
-        <v>16990.54</v>
+        <v>11065.32</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>2025-03-03</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -3268,38 +3268,38 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>3004.44</v>
+        <v>7262.6</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>2025-04-11</t>
+          <t>2025-06-12</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>31296.22</v>
+        <v>4794.65</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -3310,35 +3310,35 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>2025-04-09</t>
+          <t>2025-06-05</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>10207.4</v>
+        <v>19411.98</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>2025-05-28</t>
+          <t>2025-07-22</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -3352,21 +3352,21 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>2887.21</v>
+        <v>14370.8</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Piura</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>2025-05-13</t>
+          <t>2025-07-22</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -3380,10 +3380,10 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>38325.17</v>
+        <v>52862.4</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -3394,7 +3394,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>2025-07-12</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -3408,54 +3408,54 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>9763.76</v>
+        <v>7945.73</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>2025-06-20</t>
+          <t>2025-08-26</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>29893.33</v>
+        <v>118225.63</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>2025-06-04</t>
+          <t>2025-08-02</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -3464,10 +3464,10 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>73281.10000000001</v>
+        <v>9207.389999999999</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -3478,12 +3478,12 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>2025-06-06</t>
+          <t>2025-08-27</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -3492,10 +3492,10 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E109" s="3" t="n">
-        <v>8303.620000000001</v>
+        <v>7733.06</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -3506,68 +3506,68 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>2025-06-20</t>
+          <t>2025-09-06</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="E110" s="3" t="n">
-        <v>5344.2</v>
+        <v>13996.01</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>2025-07-03</t>
+          <t>2025-09-17</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>2895.86</v>
+        <v>27369.14</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>Trujillo</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>2025-07-06</t>
+          <t>2025-09-27</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -3576,26 +3576,26 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>167509.69</v>
+        <v>34782.82</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>Arequipa</t>
+          <t>Trujillo</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>2025-07-26</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -3604,10 +3604,10 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>56887.75</v>
+        <v>10753.95</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -3618,7 +3618,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>2025-07-12</t>
+          <t>2025-09-03</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -3632,26 +3632,26 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>4921.92</v>
+        <v>3429.95</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>2025-08-12</t>
+          <t>2025-10-22</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -3660,26 +3660,26 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>88595.39</v>
+        <v>13623.4</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Cusco</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>2025-08-12</t>
+          <t>2025-10-22</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -3688,82 +3688,82 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>44670.07</v>
+        <v>8712.93</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>2025-09-17</t>
+          <t>2025-10-27</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>12315.21</v>
+        <v>8132.45</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>2025-09-15</t>
+          <t>2025-11-05</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>150866.25</v>
+        <v>16568.42</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>2025-09-07</t>
+          <t>2025-11-02</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -3772,26 +3772,26 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>8320.75</v>
+        <v>53756.25</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>Lima</t>
+          <t>Arequipa</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>2025-09-15</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -3800,54 +3800,54 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="E120" s="3" t="n">
-        <v>9895.07</v>
+        <v>51192.12</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>2025-10-03</t>
+          <t>2025-11-27</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>Silla</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Muebles</t>
+          <t>Electrónicos</t>
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="E121" s="3" t="n">
-        <v>17674.99</v>
+        <v>14589.54</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>Cusco</t>
+          <t>Lima</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2025-12-28</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Escritorio</t>
+          <t>Silla</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -3856,10 +3856,10 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>13284.39</v>
+        <v>15692.26</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -3870,24 +3870,24 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>2025-10-08</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>Laptop</t>
+          <t>Escritorio</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>Electrónicos</t>
+          <t>Muebles</t>
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="E123" s="3" t="n">
-        <v>109433.86</v>
+        <v>49504.66</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -3898,12 +3898,12 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>2025-10-26</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Laptop</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -3912,10 +3912,10 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>23971.31</v>
+        <v>143392.41</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -3926,12 +3926,12 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>2025-10-15</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>Teclado</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
@@ -3940,238 +3940,14 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>7425.13</v>
+        <v>60308.73</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>Piura</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-10</t>
-        </is>
-      </c>
-      <c r="B126" s="2" t="inlineStr">
-        <is>
-          <t>Silla</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr">
-        <is>
-          <t>Muebles</t>
-        </is>
-      </c>
-      <c r="D126" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="E126" s="3" t="n">
-        <v>3771.58</v>
-      </c>
-      <c r="F126" s="2" t="inlineStr">
-        <is>
           <t>Trujillo</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-27</t>
-        </is>
-      </c>
-      <c r="B127" s="2" t="inlineStr">
-        <is>
-          <t>Escritorio</t>
-        </is>
-      </c>
-      <c r="C127" s="2" t="inlineStr">
-        <is>
-          <t>Muebles</t>
-        </is>
-      </c>
-      <c r="D127" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="E127" s="3" t="n">
-        <v>34509.32</v>
-      </c>
-      <c r="F127" s="2" t="inlineStr">
-        <is>
-          <t>Arequipa</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-03</t>
-        </is>
-      </c>
-      <c r="B128" s="2" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C128" s="2" t="inlineStr">
-        <is>
-          <t>Electrónicos</t>
-        </is>
-      </c>
-      <c r="D128" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="E128" s="3" t="n">
-        <v>186911.04</v>
-      </c>
-      <c r="F128" s="2" t="inlineStr">
-        <is>
-          <t>Piura</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-21</t>
-        </is>
-      </c>
-      <c r="B129" s="2" t="inlineStr">
-        <is>
-          <t>Teclado</t>
-        </is>
-      </c>
-      <c r="C129" s="2" t="inlineStr">
-        <is>
-          <t>Electrónicos</t>
-        </is>
-      </c>
-      <c r="D129" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="E129" s="3" t="n">
-        <v>13228.24</v>
-      </c>
-      <c r="F129" s="2" t="inlineStr">
-        <is>
-          <t>Arequipa</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-27</t>
-        </is>
-      </c>
-      <c r="B130" s="2" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="C130" s="2" t="inlineStr">
-        <is>
-          <t>Electrónicos</t>
-        </is>
-      </c>
-      <c r="D130" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E130" s="3" t="n">
-        <v>1664.7</v>
-      </c>
-      <c r="F130" s="2" t="inlineStr">
-        <is>
-          <t>Arequipa</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="2" t="inlineStr">
-        <is>
-          <t>2025-12-12</t>
-        </is>
-      </c>
-      <c r="B131" s="2" t="inlineStr">
-        <is>
-          <t>Laptop</t>
-        </is>
-      </c>
-      <c r="C131" s="2" t="inlineStr">
-        <is>
-          <t>Electrónicos</t>
-        </is>
-      </c>
-      <c r="D131" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="E131" s="3" t="n">
-        <v>83673.34</v>
-      </c>
-      <c r="F131" s="2" t="inlineStr">
-        <is>
-          <t>Piura</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="2" t="inlineStr">
-        <is>
-          <t>2025-12-09</t>
-        </is>
-      </c>
-      <c r="B132" s="2" t="inlineStr">
-        <is>
-          <t>Monitor</t>
-        </is>
-      </c>
-      <c r="C132" s="2" t="inlineStr">
-        <is>
-          <t>Electrónicos</t>
-        </is>
-      </c>
-      <c r="D132" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="E132" s="3" t="n">
-        <v>14652.46</v>
-      </c>
-      <c r="F132" s="2" t="inlineStr">
-        <is>
-          <t>Piura</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="2" t="inlineStr">
-        <is>
-          <t>2025-12-18</t>
-        </is>
-      </c>
-      <c r="B133" s="2" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="C133" s="2" t="inlineStr">
-        <is>
-          <t>Electrónicos</t>
-        </is>
-      </c>
-      <c r="D133" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="E133" s="3" t="n">
-        <v>9425.719999999999</v>
-      </c>
-      <c r="F133" s="2" t="inlineStr">
-        <is>
-          <t>Arequipa</t>
         </is>
       </c>
     </row>

</xml_diff>